<commit_message>
Added MID function practice and cleaned up columns
</commit_message>
<xml_diff>
--- a/Cleaned_Data_KananeloKhabane.xlsx
+++ b/Cleaned_Data_KananeloKhabane.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\T14\Desktop\M4ACE\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{C8A1668F-4723-4712-8E90-05F8710E48CB}" xr6:coauthVersionLast="36" xr6:coauthVersionMax="36" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{6A85FB9C-287A-4783-9E56-FD34206B69D2}" xr6:coauthVersionLast="36" xr6:coauthVersionMax="36" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="0" yWindow="0" windowWidth="19200" windowHeight="6810" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -18,13 +18,13 @@
   </sheets>
   <calcPr calcId="191029"/>
   <pivotCaches>
-    <pivotCache cacheId="18" r:id="rId3"/>
+    <pivotCache cacheId="0" r:id="rId3"/>
   </pivotCaches>
 </workbook>
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="79" uniqueCount="56">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="80" uniqueCount="57">
   <si>
     <t xml:space="preserve">JUAREZ, JOSE </t>
   </si>
@@ -134,9 +134,6 @@
     <t xml:space="preserve">FALLENGRANO, BILL </t>
   </si>
   <si>
-    <t>Employee Name</t>
-  </si>
-  <si>
     <t>Hire Date</t>
   </si>
   <si>
@@ -158,24 +155,6 @@
     <t>Full Names</t>
   </si>
   <si>
-    <t>Employee Name2</t>
-  </si>
-  <si>
-    <t>Column3</t>
-  </si>
-  <si>
-    <t>Column1</t>
-  </si>
-  <si>
-    <t>Column2</t>
-  </si>
-  <si>
-    <t>Column4</t>
-  </si>
-  <si>
-    <t>Column5</t>
-  </si>
-  <si>
     <t>Sum of Salary</t>
   </si>
   <si>
@@ -192,6 +171,30 @@
   </si>
   <si>
     <t>Sales</t>
+  </si>
+  <si>
+    <t>Raw dept. data</t>
+  </si>
+  <si>
+    <t>CON_function</t>
+  </si>
+  <si>
+    <t>Raw Title data</t>
+  </si>
+  <si>
+    <t>Raw_Full names</t>
+  </si>
+  <si>
+    <t>Proper_Function</t>
+  </si>
+  <si>
+    <t>Find_function</t>
+  </si>
+  <si>
+    <t>Length_function</t>
+  </si>
+  <si>
+    <t>MID_function</t>
   </si>
 </sst>
 </file>
@@ -915,33 +918,7 @@
           </a:effectLst>
         </c:spPr>
         <c:marker>
-          <c:symbol val="circle"/>
-          <c:size val="6"/>
-          <c:spPr>
-            <a:gradFill>
-              <a:gsLst>
-                <a:gs pos="0">
-                  <a:schemeClr val="accent1"/>
-                </a:gs>
-                <a:gs pos="100000">
-                  <a:schemeClr val="accent1">
-                    <a:lumMod val="84000"/>
-                  </a:schemeClr>
-                </a:gs>
-              </a:gsLst>
-              <a:lin ang="5400000" scaled="1"/>
-            </a:gradFill>
-            <a:ln>
-              <a:noFill/>
-            </a:ln>
-            <a:effectLst>
-              <a:outerShdw blurRad="76200" dir="18900000" sy="23000" kx="-1200000" algn="bl" rotWithShape="0">
-                <a:prstClr val="black">
-                  <a:alpha val="20000"/>
-                </a:prstClr>
-              </a:outerShdw>
-            </a:effectLst>
-          </c:spPr>
+          <c:symbol val="none"/>
         </c:marker>
         <c:dLbl>
           <c:idx val="0"/>
@@ -2313,7 +2290,7 @@
 </file>
 
 <file path=xl/pivotTables/pivotTable1.xml><?xml version="1.0" encoding="utf-8"?>
-<pivotTableDefinition xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="xr" xr:uid="{4514A0FA-BE04-459B-92A5-CE47C87CA485}" name="PivotTable15" cacheId="18" applyNumberFormats="0" applyBorderFormats="0" applyFontFormats="0" applyPatternFormats="0" applyAlignmentFormats="0" applyWidthHeightFormats="1" dataCaption="Values" updatedVersion="6" minRefreshableVersion="3" useAutoFormatting="1" rowGrandTotals="0" colGrandTotals="0" itemPrintTitles="1" createdVersion="6" indent="0" compact="0" compactData="0" multipleFieldFilters="0" chartFormat="1">
+<pivotTableDefinition xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="xr" xr:uid="{4514A0FA-BE04-459B-92A5-CE47C87CA485}" name="PivotTable15" cacheId="0" applyNumberFormats="0" applyBorderFormats="0" applyFontFormats="0" applyPatternFormats="0" applyAlignmentFormats="0" applyWidthHeightFormats="1" dataCaption="Values" updatedVersion="6" minRefreshableVersion="3" useAutoFormatting="1" rowGrandTotals="0" colGrandTotals="0" itemPrintTitles="1" createdVersion="6" indent="0" compact="0" compactData="0" multipleFieldFilters="0" chartFormat="1">
   <location ref="A3:B9" firstHeaderRow="1" firstDataRow="1" firstDataCol="1"/>
   <pivotFields count="14">
     <pivotField compact="0" outline="0" showAll="0" defaultSubtotal="0">
@@ -2482,14 +2459,14 @@
     <sortCondition descending="1" ref="J1:J20"/>
   </sortState>
   <tableColumns count="14">
-    <tableColumn id="1" xr3:uid="{00000000-0010-0000-0000-000001000000}" name="Employee Name"/>
-    <tableColumn id="2" xr3:uid="{00000000-0010-0000-0000-000002000000}" name="Employee Name2">
+    <tableColumn id="1" xr3:uid="{00000000-0010-0000-0000-000001000000}" name="Raw_Full names"/>
+    <tableColumn id="2" xr3:uid="{00000000-0010-0000-0000-000002000000}" name="Proper_Function">
       <calculatedColumnFormula>PROPER(A2)</calculatedColumnFormula>
     </tableColumn>
-    <tableColumn id="3" xr3:uid="{00000000-0010-0000-0000-000003000000}" name="Column5">
+    <tableColumn id="3" xr3:uid="{00000000-0010-0000-0000-000003000000}" name="Find_function">
       <calculatedColumnFormula>FIND(",",B2)</calculatedColumnFormula>
     </tableColumn>
-    <tableColumn id="4" xr3:uid="{00000000-0010-0000-0000-000004000000}" name="Column3">
+    <tableColumn id="4" xr3:uid="{00000000-0010-0000-0000-000004000000}" name="Length_function">
       <calculatedColumnFormula>LEN(B2)</calculatedColumnFormula>
     </tableColumn>
     <tableColumn id="5" xr3:uid="{00000000-0010-0000-0000-000005000000}" name="First Name">
@@ -2498,7 +2475,7 @@
     <tableColumn id="6" xr3:uid="{00000000-0010-0000-0000-000006000000}" name="Last Name">
       <calculatedColumnFormula>LEFT(B2,C2-1)</calculatedColumnFormula>
     </tableColumn>
-    <tableColumn id="7" xr3:uid="{00000000-0010-0000-0000-000007000000}" name="Column4">
+    <tableColumn id="7" xr3:uid="{00000000-0010-0000-0000-000007000000}" name="CON_function">
       <calculatedColumnFormula>CONCATENATE(E2," ",F2)</calculatedColumnFormula>
     </tableColumn>
     <tableColumn id="8" xr3:uid="{00000000-0010-0000-0000-000008000000}" name="Full Names">
@@ -2506,11 +2483,11 @@
     </tableColumn>
     <tableColumn id="9" xr3:uid="{00000000-0010-0000-0000-000009000000}" name="Hire Date" dataDxfId="3"/>
     <tableColumn id="10" xr3:uid="{00000000-0010-0000-0000-00000A000000}" name="Salary" dataDxfId="2" dataCellStyle="Currency"/>
-    <tableColumn id="11" xr3:uid="{00000000-0010-0000-0000-00000B000000}" name="Column2"/>
+    <tableColumn id="11" xr3:uid="{00000000-0010-0000-0000-00000B000000}" name="Raw dept. data"/>
     <tableColumn id="12" xr3:uid="{00000000-0010-0000-0000-00000C000000}" name="Department" dataDxfId="1">
       <calculatedColumnFormula>SUBSTITUTE(PROPER(K2),"Mktg","Marketing")</calculatedColumnFormula>
     </tableColumn>
-    <tableColumn id="13" xr3:uid="{00000000-0010-0000-0000-00000D000000}" name="Column1"/>
+    <tableColumn id="13" xr3:uid="{00000000-0010-0000-0000-00000D000000}" name="Raw Title data"/>
     <tableColumn id="14" xr3:uid="{00000000-0010-0000-0000-00000E000000}" name="Job Title" dataDxfId="0">
       <calculatedColumnFormula>SUBSTITUTE(PROPER(M2),"Vp","Vice President")</calculatedColumnFormula>
     </tableColumn>
@@ -2816,68 +2793,72 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:N22"/>
+  <dimension ref="A1:P22"/>
   <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
   <cols>
     <col min="1" max="1" width="20.54296875" hidden="1" customWidth="1"/>
-    <col min="2" max="2" width="17.26953125" hidden="1" customWidth="1"/>
+    <col min="2" max="2" width="17.26953125" customWidth="1"/>
     <col min="3" max="4" width="18.54296875" hidden="1" customWidth="1"/>
     <col min="5" max="6" width="18.54296875" customWidth="1"/>
     <col min="7" max="7" width="18.54296875" hidden="1" customWidth="1"/>
     <col min="8" max="8" width="18.54296875" customWidth="1"/>
     <col min="9" max="9" width="16.08984375" style="2" customWidth="1"/>
     <col min="10" max="10" width="16.7265625" style="1" customWidth="1"/>
-    <col min="11" max="11" width="14.81640625" hidden="1" customWidth="1"/>
+    <col min="11" max="11" width="10.26953125" hidden="1" customWidth="1"/>
     <col min="12" max="12" width="17.26953125" customWidth="1"/>
     <col min="13" max="13" width="7.08984375" hidden="1" customWidth="1"/>
     <col min="14" max="14" width="21.453125" customWidth="1"/>
+    <col min="16" max="16" width="0" hidden="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:14" s="4" customFormat="1" ht="17" x14ac:dyDescent="0.5">
+    <row r="1" spans="1:16" s="4" customFormat="1" ht="17" x14ac:dyDescent="0.5">
       <c r="A1" s="4" t="s">
+        <v>52</v>
+      </c>
+      <c r="B1" s="4" t="s">
+        <v>53</v>
+      </c>
+      <c r="C1" s="4" t="s">
+        <v>54</v>
+      </c>
+      <c r="D1" s="4" t="s">
+        <v>55</v>
+      </c>
+      <c r="E1" s="4" t="s">
+        <v>40</v>
+      </c>
+      <c r="F1" s="4" t="s">
+        <v>41</v>
+      </c>
+      <c r="G1" s="4" t="s">
+        <v>50</v>
+      </c>
+      <c r="H1" s="4" t="s">
+        <v>42</v>
+      </c>
+      <c r="I1" s="5" t="s">
         <v>36</v>
       </c>
-      <c r="B1" s="4" t="s">
-        <v>44</v>
-      </c>
-      <c r="C1" s="4" t="s">
+      <c r="J1" s="6" t="s">
+        <v>37</v>
+      </c>
+      <c r="K1" s="4" t="s">
         <v>49</v>
       </c>
-      <c r="D1" s="4" t="s">
-        <v>45</v>
-      </c>
-      <c r="E1" s="4" t="s">
-        <v>41</v>
-      </c>
-      <c r="F1" s="4" t="s">
-        <v>42</v>
-      </c>
-      <c r="G1" s="4" t="s">
-        <v>48</v>
-      </c>
-      <c r="H1" s="4" t="s">
-        <v>43</v>
-      </c>
-      <c r="I1" s="5" t="s">
-        <v>37</v>
-      </c>
-      <c r="J1" s="6" t="s">
+      <c r="L1" s="4" t="s">
         <v>38</v>
       </c>
-      <c r="K1" s="4" t="s">
-        <v>47</v>
-      </c>
-      <c r="L1" s="4" t="s">
+      <c r="M1" s="4" t="s">
+        <v>51</v>
+      </c>
+      <c r="N1" s="4" t="s">
         <v>39</v>
       </c>
-      <c r="M1" s="4" t="s">
-        <v>46</v>
-      </c>
-      <c r="N1" s="4" t="s">
-        <v>40</v>
+      <c r="P1" s="4" t="s">
+        <v>56</v>
       </c>
     </row>
-    <row r="2" spans="1:14" x14ac:dyDescent="0.35">
+    <row r="2" spans="1:16" x14ac:dyDescent="0.35">
       <c r="A2" t="s">
         <v>27</v>
       </c>
@@ -2929,8 +2910,12 @@
         <f t="shared" ref="N2:N20" si="8">SUBSTITUTE(PROPER(M2),"Vp","Vice President")</f>
         <v>Vice President</v>
       </c>
+      <c r="P2" t="str">
+        <f>MID(F3,3,5)</f>
+        <v>lleng</v>
+      </c>
     </row>
-    <row r="3" spans="1:14" x14ac:dyDescent="0.35">
+    <row r="3" spans="1:16" x14ac:dyDescent="0.35">
       <c r="A3" t="s">
         <v>35</v>
       </c>
@@ -2983,7 +2968,7 @@
         <v>Senior Administrator</v>
       </c>
     </row>
-    <row r="4" spans="1:14" x14ac:dyDescent="0.35">
+    <row r="4" spans="1:16" x14ac:dyDescent="0.35">
       <c r="A4" t="s">
         <v>26</v>
       </c>
@@ -3036,7 +3021,7 @@
         <v>Cost Accountant</v>
       </c>
     </row>
-    <row r="5" spans="1:14" x14ac:dyDescent="0.35">
+    <row r="5" spans="1:16" x14ac:dyDescent="0.35">
       <c r="A5" t="s">
         <v>34</v>
       </c>
@@ -3089,7 +3074,7 @@
         <v>Cost Accountant</v>
       </c>
     </row>
-    <row r="6" spans="1:14" x14ac:dyDescent="0.35">
+    <row r="6" spans="1:16" x14ac:dyDescent="0.35">
       <c r="A6" t="s">
         <v>12</v>
       </c>
@@ -3142,7 +3127,7 @@
         <v>Cost Accountant</v>
       </c>
     </row>
-    <row r="7" spans="1:14" x14ac:dyDescent="0.35">
+    <row r="7" spans="1:16" x14ac:dyDescent="0.35">
       <c r="A7" t="s">
         <v>10</v>
       </c>
@@ -3195,7 +3180,7 @@
         <v>Manager</v>
       </c>
     </row>
-    <row r="8" spans="1:14" x14ac:dyDescent="0.35">
+    <row r="8" spans="1:16" x14ac:dyDescent="0.35">
       <c r="A8" t="s">
         <v>15</v>
       </c>
@@ -3248,7 +3233,7 @@
         <v>Designer</v>
       </c>
     </row>
-    <row r="9" spans="1:14" x14ac:dyDescent="0.35">
+    <row r="9" spans="1:16" x14ac:dyDescent="0.35">
       <c r="A9" t="s">
         <v>30</v>
       </c>
@@ -3301,7 +3286,7 @@
         <v>Team Leader</v>
       </c>
     </row>
-    <row r="10" spans="1:14" x14ac:dyDescent="0.35">
+    <row r="10" spans="1:16" x14ac:dyDescent="0.35">
       <c r="A10" t="s">
         <v>33</v>
       </c>
@@ -3354,7 +3339,7 @@
         <v>Intern</v>
       </c>
     </row>
-    <row r="11" spans="1:14" x14ac:dyDescent="0.35">
+    <row r="11" spans="1:16" x14ac:dyDescent="0.35">
       <c r="A11" t="s">
         <v>18</v>
       </c>
@@ -3407,7 +3392,7 @@
         <v>Sales Executive</v>
       </c>
     </row>
-    <row r="12" spans="1:14" x14ac:dyDescent="0.35">
+    <row r="12" spans="1:16" x14ac:dyDescent="0.35">
       <c r="A12" t="s">
         <v>24</v>
       </c>
@@ -3460,7 +3445,7 @@
         <v>Senior Technician</v>
       </c>
     </row>
-    <row r="13" spans="1:14" x14ac:dyDescent="0.35">
+    <row r="13" spans="1:16" x14ac:dyDescent="0.35">
       <c r="A13" t="s">
         <v>0</v>
       </c>
@@ -3489,7 +3474,7 @@
         <v xml:space="preserve"> Jose  Juarez</v>
       </c>
       <c r="H13" t="str">
-        <f>TRIM(G13)</f>
+        <f t="shared" ref="H13:H20" si="9">TRIM(G13)</f>
         <v>Jose Juarez</v>
       </c>
       <c r="I13" s="3">
@@ -3513,7 +3498,7 @@
         <v>Intern</v>
       </c>
     </row>
-    <row r="14" spans="1:14" x14ac:dyDescent="0.35">
+    <row r="14" spans="1:16" x14ac:dyDescent="0.35">
       <c r="A14" t="s">
         <v>21</v>
       </c>
@@ -3542,7 +3527,7 @@
         <v xml:space="preserve"> Tammy  Bursteyn</v>
       </c>
       <c r="H14" t="str">
-        <f>TRIM(G14)</f>
+        <f t="shared" si="9"/>
         <v>Tammy Bursteyn</v>
       </c>
       <c r="I14" s="3">
@@ -3566,7 +3551,7 @@
         <v>Sales Executive</v>
       </c>
     </row>
-    <row r="15" spans="1:14" x14ac:dyDescent="0.35">
+    <row r="15" spans="1:16" x14ac:dyDescent="0.35">
       <c r="A15" t="s">
         <v>6</v>
       </c>
@@ -3595,7 +3580,7 @@
         <v xml:space="preserve"> Sarah Baker</v>
       </c>
       <c r="H15" t="str">
-        <f>TRIM(G15)</f>
+        <f t="shared" si="9"/>
         <v>Sarah Baker</v>
       </c>
       <c r="I15" s="3">
@@ -3619,7 +3604,7 @@
         <v>Sales Executive</v>
       </c>
     </row>
-    <row r="16" spans="1:14" x14ac:dyDescent="0.35">
+    <row r="16" spans="1:16" x14ac:dyDescent="0.35">
       <c r="A16" t="s">
         <v>22</v>
       </c>
@@ -3648,7 +3633,7 @@
         <v xml:space="preserve"> Bobby Busser</v>
       </c>
       <c r="H16" t="str">
-        <f>TRIM(G16)</f>
+        <f t="shared" si="9"/>
         <v>Bobby Busser</v>
       </c>
       <c r="I16" s="3">
@@ -3701,7 +3686,7 @@
         <v xml:space="preserve"> Johnny  Abraham</v>
       </c>
       <c r="H17" t="str">
-        <f>TRIM(G17)</f>
+        <f t="shared" si="9"/>
         <v>Johnny Abraham</v>
       </c>
       <c r="I17" s="3">
@@ -3754,7 +3739,7 @@
         <v xml:space="preserve"> Billy Balotelli</v>
       </c>
       <c r="H18" t="str">
-        <f>TRIM(G18)</f>
+        <f t="shared" si="9"/>
         <v>Billy Balotelli</v>
       </c>
       <c r="I18" s="3">
@@ -3807,7 +3792,7 @@
         <v xml:space="preserve"> Jane  Doe</v>
       </c>
       <c r="H19" t="str">
-        <f>TRIM(G19)</f>
+        <f t="shared" si="9"/>
         <v>Jane Doe</v>
       </c>
       <c r="I19" s="3">
@@ -3860,7 +3845,7 @@
         <v xml:space="preserve"> Tom  Bursteyn </v>
       </c>
       <c r="H20" t="str">
-        <f>TRIM(G20)</f>
+        <f t="shared" si="9"/>
         <v>Tom Bursteyn</v>
       </c>
       <c r="I20" s="3">
@@ -3910,15 +3895,15 @@
   <sheetData>
     <row r="3" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A3" s="7" t="s">
-        <v>39</v>
+        <v>38</v>
       </c>
       <c r="B3" t="s">
-        <v>50</v>
+        <v>43</v>
       </c>
     </row>
     <row r="4" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A4" t="s">
-        <v>51</v>
+        <v>44</v>
       </c>
       <c r="B4" s="8">
         <v>79950</v>
@@ -3926,7 +3911,7 @@
     </row>
     <row r="5" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A5" t="s">
-        <v>52</v>
+        <v>45</v>
       </c>
       <c r="B5" s="8">
         <v>85000</v>
@@ -3934,7 +3919,7 @@
     </row>
     <row r="6" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A6" t="s">
-        <v>53</v>
+        <v>46</v>
       </c>
       <c r="B6" s="8">
         <v>251750</v>
@@ -3942,7 +3927,7 @@
     </row>
     <row r="7" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A7" t="s">
-        <v>54</v>
+        <v>47</v>
       </c>
       <c r="B7" s="8">
         <v>46000</v>
@@ -3958,7 +3943,7 @@
     </row>
     <row r="9" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A9" t="s">
-        <v>55</v>
+        <v>48</v>
       </c>
       <c r="B9" s="8">
         <v>233500</v>

</xml_diff>